<commit_message>
docs: add graphics clockify
</commit_message>
<xml_diff>
--- a/docs/Sprint 3/deliverables/10-S3-dedication.xlsx
+++ b/docs/Sprint 3/deliverables/10-S3-dedication.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4700CC28-6D58-4809-94E4-E5B6CB49B7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{02C8C9D8-2F21-45BA-9A66-91BB45160C54}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="4" xr2:uid="{02C8C9D8-2F21-45BA-9A66-91BB45160C54}"/>
   </bookViews>
   <sheets>
     <sheet name="Contribución a los entregables" sheetId="1" r:id="rId1"/>
@@ -440,6 +440,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="46" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="46" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -451,15 +460,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="46" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="46" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1767,34 +1767,34 @@
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B33" s="23" t="s">
+      <c r="B33" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="C33" s="23"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="23"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="23"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="26"/>
+      <c r="F33" s="26"/>
+      <c r="G33" s="26"/>
     </row>
     <row r="34" spans="2:7" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="23" t="s">
+      <c r="B34" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="C34" s="23"/>
-      <c r="D34" s="23"/>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="23"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="26"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="26"/>
     </row>
     <row r="35" spans="2:7" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="23" t="s">
+      <c r="B35" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="C35" s="23"/>
-      <c r="D35" s="23"/>
-      <c r="E35" s="23"/>
-      <c r="F35" s="23"/>
-      <c r="G35" s="23"/>
+      <c r="C35" s="26"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
+      <c r="F35" s="26"/>
+      <c r="G35" s="26"/>
     </row>
     <row r="36" spans="2:7" ht="44.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
@@ -1845,11 +1845,11 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" ht="101.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E3" s="11"/>
@@ -2498,11 +2498,11 @@
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
       <c r="H28" s="6">
         <f>SUM(H2:H21)/20</f>
         <v>1.0000000000000002</v>
@@ -2633,7 +2633,7 @@
       <c r="C2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="26">
+      <c r="D2" s="22">
         <v>1.3212152777777777</v>
       </c>
       <c r="E2" s="17">
@@ -2659,7 +2659,7 @@
       <c r="C3" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="27">
+      <c r="D3" s="23">
         <v>0.87565972222222221</v>
       </c>
       <c r="E3" s="17">
@@ -2685,7 +2685,7 @@
       <c r="C4" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="28">
+      <c r="D4" s="24">
         <v>1.0733333333333333</v>
       </c>
       <c r="E4" s="17">
@@ -2711,7 +2711,7 @@
       <c r="C5" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="27">
+      <c r="D5" s="23">
         <v>0.79408564814814819</v>
       </c>
       <c r="E5" s="17">
@@ -2737,7 +2737,7 @@
       <c r="C6" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="27">
+      <c r="D6" s="23">
         <v>0.91697916666666668</v>
       </c>
       <c r="E6" s="17">
@@ -2763,7 +2763,7 @@
       <c r="C7" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="27">
+      <c r="D7" s="23">
         <v>0.9202893518518519</v>
       </c>
       <c r="E7" s="17">
@@ -2790,7 +2790,7 @@
       <c r="C8" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="27">
+      <c r="D8" s="23">
         <v>0.97291666666666665</v>
       </c>
       <c r="E8" s="17">
@@ -2816,7 +2816,7 @@
       <c r="C9" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="27">
+      <c r="D9" s="23">
         <v>0.76469907407407411</v>
       </c>
       <c r="E9" s="17">
@@ -2842,7 +2842,7 @@
       <c r="C10" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="27">
+      <c r="D10" s="23">
         <v>0.81597222222222221</v>
       </c>
       <c r="E10" s="17">
@@ -2868,7 +2868,7 @@
       <c r="C11" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="27">
+      <c r="D11" s="23">
         <v>0.83481481481481479</v>
       </c>
       <c r="E11" s="17">
@@ -2894,7 +2894,7 @@
       <c r="C12" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="27">
+      <c r="D12" s="23">
         <v>0.75748842592592591</v>
       </c>
       <c r="E12" s="17">
@@ -2920,7 +2920,7 @@
       <c r="C13" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="27">
+      <c r="D13" s="23">
         <v>0.875</v>
       </c>
       <c r="E13" s="17">
@@ -2946,7 +2946,7 @@
       <c r="C14" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="27">
+      <c r="D14" s="23">
         <v>0.93865740740740744</v>
       </c>
       <c r="E14" s="17">
@@ -2973,7 +2973,7 @@
       <c r="C15" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="28">
+      <c r="D15" s="24">
         <v>1.0462615740740742</v>
       </c>
       <c r="E15" s="17">
@@ -2999,7 +2999,7 @@
       <c r="C16" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="27">
+      <c r="D16" s="23">
         <v>0.7492361111111111</v>
       </c>
       <c r="E16" s="17">
@@ -3025,7 +3025,7 @@
       <c r="C17" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="27">
+      <c r="D17" s="23">
         <v>0.80880787037037039</v>
       </c>
       <c r="E17" s="17">
@@ -3051,7 +3051,7 @@
       <c r="C18" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="27">
+      <c r="D18" s="23">
         <v>0.95706018518518521</v>
       </c>
       <c r="E18" s="17">
@@ -3077,7 +3077,7 @@
       <c r="C19" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="D19" s="27">
+      <c r="D19" s="23">
         <v>0.79861111111111116</v>
       </c>
       <c r="E19" s="17">
@@ -3103,7 +3103,7 @@
       <c r="C20" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="27">
+      <c r="D20" s="23">
         <v>0.84755787037037034</v>
       </c>
       <c r="E20" s="17">
@@ -3129,7 +3129,7 @@
       <c r="C21" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="27">
+      <c r="D21" s="23">
         <v>0.75665509259259256</v>
       </c>
       <c r="E21" s="17">
@@ -3212,11 +3212,11 @@
       <c r="H27" s="2"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
       <c r="H28" s="6">
         <f>SUM(H2:H21)/20</f>
         <v>1.0000000000000004</v>
@@ -3309,9 +3309,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3477,19 +3480,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D0D844A-E87E-42E2-B155-132CABE67861}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F4B272D-551A-4AF9-B220-C688C9745ED1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3513,9 +3512,10 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F4B272D-551A-4AF9-B220-C688C9745ED1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D0D844A-E87E-42E2-B155-132CABE67861}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>